<commit_message>
renamed srs, add checklists, update test case populated, removed muda from manageuser
</commit_message>
<xml_diff>
--- a/Task 5-8/HV_Test_Case_Populated.xlsx
+++ b/Task 5-8/HV_Test_Case_Populated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 5-8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C212FBDF-E484-4EDF-8D33-58DF3B8462D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF85EB3-655D-4267-B3AD-2BF3082B8A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="879">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="877">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -2603,9 +2603,6 @@
     <t>Comments added to complex logic</t>
   </si>
   <si>
-    <t>Concern</t>
-  </si>
-  <si>
     <t>Some comments exist, but checking suffix logic, duplicate ticket logic, and JWT active-user recheck need clearer comments.</t>
   </si>
   <si>
@@ -2627,12 +2624,6 @@
     <t>Checked unit test coverage</t>
   </si>
   <si>
-    <t>Recorded</t>
-  </si>
-  <si>
-    <t>JaCoCo total code coverage = 37.30%. Recommend increasing to at least 60%-70%.</t>
-  </si>
-  <si>
     <t>Test situations documented</t>
   </si>
   <si>
@@ -2679,6 +2670,9 @@
   </si>
   <si>
     <t>consistent ui across screens</t>
+  </si>
+  <si>
+    <t>JaCoCo total code coverage = 37.30%</t>
   </si>
 </sst>
 </file>
@@ -2712,7 +2706,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2742,11 +2736,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -2814,7 +2803,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2829,13 +2818,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2843,13 +2833,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3163,13 +3146,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -5431,34 +5414,34 @@
       <c r="B4" s="5">
         <v>34</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="8">
         <v>0</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="9">
         <v>0</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="10">
         <v>0</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="10">
         <v>0</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="7">
         <v>34</v>
       </c>
     </row>
@@ -5769,7 +5752,7 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -6413,34 +6396,34 @@
       <c r="B4" s="5">
         <v>15</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="8">
         <v>0</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="9">
         <v>0</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="10">
         <v>0</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="10">
         <v>1</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="7">
         <v>16</v>
       </c>
     </row>
@@ -6876,7 +6859,7 @@
       <c r="E22" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="6" t="s">
         <v>671</v>
       </c>
       <c r="G22" s="1"/>
@@ -6924,7 +6907,7 @@
       <c r="A3" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -6935,34 +6918,34 @@
       <c r="B4" s="5">
         <v>24</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="8">
         <v>0</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="F4" s="14">
+      <c r="F4" s="9">
         <v>0</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="10">
         <v>0</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="7" t="s">
         <v>399</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="10">
         <v>2</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="K4" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="7">
         <v>26</v>
       </c>
     </row>
@@ -7286,7 +7269,7 @@
         <v>733</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>734</v>
@@ -7604,7 +7587,7 @@
       <c r="E30" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="6" t="s">
         <v>671</v>
       </c>
       <c r="G30" s="1"/>
@@ -7628,7 +7611,7 @@
       <c r="E31" s="1" t="s">
         <v>802</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="6" t="s">
         <v>671</v>
       </c>
       <c r="G31" s="1"/>
@@ -7680,13 +7663,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>809</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="14"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -7823,16 +7806,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>829</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -8034,7 +8017,7 @@
         <v>836</v>
       </c>
       <c r="C13" s="1">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
@@ -8088,7 +8071,7 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1">
         <f>C13/H13 * 100</f>
-        <v>88.157894736842096</v>
+        <v>96.05263157894737</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>838</v>
@@ -8163,11 +8146,11 @@
       <c r="B3" s="1" t="s">
         <v>849</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>853</v>
+      <c r="C3" s="5" t="s">
+        <v>413</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -8195,7 +8178,7 @@
         <v>413</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -8203,13 +8186,13 @@
         <v>846</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>855</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>853</v>
+        <v>854</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>413</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -8217,13 +8200,13 @@
         <v>353</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>856</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -8231,13 +8214,13 @@
         <v>353</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>857</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>858</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>859</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -8245,13 +8228,13 @@
         <v>353</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>860</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>861</v>
+        <v>859</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>413</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>862</v>
+        <v>876</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -8259,13 +8242,13 @@
         <v>366</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -8273,13 +8256,13 @@
         <v>366</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -8287,13 +8270,13 @@
         <v>375</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -8301,13 +8284,13 @@
         <v>375</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -8315,13 +8298,13 @@
         <v>375</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -8329,13 +8312,13 @@
         <v>375</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update test coverage in docs
</commit_message>
<xml_diff>
--- a/Task 5-8/HV_Test_Case_Populated.xlsx
+++ b/Task 5-8/HV_Test_Case_Populated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 5-8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF85EB3-655D-4267-B3AD-2BF3082B8A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4F3EB0-5200-437A-A94B-CE82AD50E0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2540,9 +2540,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Release 1 includes 3 modules: Module1, Module2, Module3. Results are based on static code review on 22/07/2026. Runtime-dependent cases remain Untested. Backend JaCoCo total coverage: 37.30%.</t>
-  </si>
-  <si>
     <t>Module code</t>
   </si>
   <si>
@@ -2673,6 +2670,9 @@
   </si>
   <si>
     <t>JaCoCo total code coverage = 37.30%</t>
+  </si>
+  <si>
+    <t>Release 1 includes 3 modules: Module1, Module2, Module3. Results are based on static code review on 22/07/2026. Runtime-dependent cases remain Untested. Backend JaCoCo total coverage: 70.66%.</t>
   </si>
 </sst>
 </file>
@@ -5752,7 +5752,7 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7269,7 +7269,7 @@
         <v>733</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>734</v>
@@ -7888,7 +7888,7 @@
         <v>831</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>832</v>
+        <v>876</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -7912,13 +7912,13 @@
         <v>812</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>832</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>833</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>834</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>397</v>
@@ -7930,7 +7930,7 @@
         <v>399</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -8014,7 +8014,7 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C13" s="1">
         <v>73</v>
@@ -8048,25 +8048,25 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1">
         <v>100</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1">
@@ -8074,12 +8074,12 @@
         <v>96.05263157894737</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -8113,86 +8113,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>841</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>842</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>843</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>844</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>845</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>846</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>847</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>848</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>850</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>852</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>853</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -8200,13 +8200,13 @@
         <v>353</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>854</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>855</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>856</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -8214,13 +8214,13 @@
         <v>353</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>856</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>857</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>858</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -8228,13 +8228,13 @@
         <v>353</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -8242,13 +8242,13 @@
         <v>366</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>860</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -8256,13 +8256,13 @@
         <v>366</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>862</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -8270,13 +8270,13 @@
         <v>375</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -8284,13 +8284,13 @@
         <v>375</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -8298,13 +8298,13 @@
         <v>375</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>866</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -8312,13 +8312,13 @@
         <v>375</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>868</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update srs with missing unit tests from frontend
</commit_message>
<xml_diff>
--- a/Task 5-8/HV_Test_Case_Populated.xlsx
+++ b/Task 5-8/HV_Test_Case_Populated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 5-8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4F3EB0-5200-437A-A94B-CE82AD50E0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD169FCB-9ADD-40EF-ADEE-26ADF06CE456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="877">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1417" uniqueCount="880">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -2669,10 +2669,19 @@
     <t>consistent ui across screens</t>
   </si>
   <si>
-    <t>JaCoCo total code coverage = 37.30%</t>
-  </si>
-  <si>
     <t>Release 1 includes 3 modules: Module1, Module2, Module3. Results are based on static code review on 22/07/2026. Runtime-dependent cases remain Untested. Backend JaCoCo total coverage: 70.66%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1.2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">M </t>
+  </si>
+  <si>
+    <t>Add controller + SocialAuth + AuthProvider tests; JaCoCo 37.30% → 70.66%; N+1 fix (JOIN FETCH) in getUserHistory</t>
+  </si>
+  <si>
+    <t>JaCoCo total code coverage = 70.66%</t>
   </si>
 </sst>
 </file>
@@ -2803,7 +2812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2833,6 +2842,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3135,7 +3151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3302,6 +3318,21 @@
       <c r="E14" s="1" t="s">
         <v>25</v>
       </c>
+    </row>
+    <row r="15" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" s="15">
+        <v>46030</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>876</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>877</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>878</v>
+      </c>
+      <c r="E15" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7888,7 +7919,7 @@
         <v>831</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -8234,7 +8265,7 @@
         <v>413</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
remove waste, update srs, update docs, fix N+1 problem
</commit_message>
<xml_diff>
--- a/Task 5-8/HV_Test_Case_Populated.xlsx
+++ b/Task 5-8/HV_Test_Case_Populated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kohaku\Downloads\LAB301\Task 5-8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD169FCB-9ADD-40EF-ADEE-26ADF06CE456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A9CD5C-E868-4DB8-A504-5022E52A7542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2247,9 +2247,6 @@
     <t>Response &lt; 500ms. All results correct.</t>
   </si>
   <si>
-    <t>Performance must be measured at runtime. Duplicate-check query runs per ticket.</t>
-  </si>
-  <si>
     <t>F3-13</t>
   </si>
   <si>
@@ -2663,15 +2660,9 @@
     <t>most unused codes removed.</t>
   </si>
   <si>
-    <t>Core screens implemented. Optional preview, AdSense, and gamification are not implemented. But they were also never planned in the srs</t>
-  </si>
-  <si>
     <t>consistent ui across screens</t>
   </si>
   <si>
-    <t>Release 1 includes 3 modules: Module1, Module2, Module3. Results are based on static code review on 22/07/2026. Runtime-dependent cases remain Untested. Backend JaCoCo total coverage: 70.66%.</t>
-  </si>
-  <si>
     <t xml:space="preserve">v1.2 </t>
   </si>
   <si>
@@ -2682,6 +2673,15 @@
   </si>
   <si>
     <t>JaCoCo total code coverage = 70.66%</t>
+  </si>
+  <si>
+    <t>Backend JaCoCo total coverage: 70.66%.</t>
+  </si>
+  <si>
+    <t>Duplicate checking for authenticated users uses a single batch query with an IN clause.</t>
+  </si>
+  <si>
+    <t>Optional stretch goals from the SRS: Preview ticket, AdSense, and gamification comments were not implemented and are marked N/A.</t>
   </si>
 </sst>
 </file>
@@ -2812,7 +2812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2837,18 +2837,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3162,13 +3159,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -3320,17 +3317,17 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A15" s="15">
+      <c r="A15" s="12">
         <v>46030</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>876</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>877</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>878</v>
+        <v>873</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>874</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>875</v>
       </c>
       <c r="E15" s="7"/>
     </row>
@@ -5783,7 +5780,7 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -7300,7 +7297,7 @@
         <v>733</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>734</v>
@@ -7313,21 +7310,21 @@
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1" t="s">
-        <v>735</v>
+        <v>878</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>737</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>738</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>739</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>694</v>
@@ -7339,21 +7336,21 @@
         <v>8</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
+        <v>740</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>741</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>742</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>743</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>744</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>412</v>
@@ -7365,24 +7362,24 @@
         <v>8</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>746</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>747</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>748</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>749</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>750</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>413</v>
@@ -7391,24 +7388,24 @@
         <v>8</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>752</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>753</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>754</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>755</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>756</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>413</v>
@@ -7417,24 +7414,24 @@
         <v>8</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>260</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>759</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>760</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>761</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>413</v>
@@ -7443,24 +7440,24 @@
         <v>8</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>263</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>764</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="E24" s="1" t="s">
         <v>765</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>766</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>413</v>
@@ -7469,24 +7466,24 @@
         <v>8</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
+        <v>767</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>768</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>769</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>770</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="E25" s="1" t="s">
         <v>771</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>772</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>413</v>
@@ -7495,24 +7492,24 @@
         <v>8</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>270</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>775</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="E26" s="1" t="s">
         <v>776</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>777</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>413</v>
@@ -7521,24 +7518,24 @@
         <v>8</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>779</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>780</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>781</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="E27" s="1" t="s">
         <v>782</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>783</v>
       </c>
       <c r="F27" s="5" t="s">
         <v>413</v>
@@ -7547,24 +7544,24 @@
         <v>8</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
+        <v>784</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>785</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>786</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>787</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>788</v>
-      </c>
       <c r="E28" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="F28" s="5" t="s">
         <v>413</v>
@@ -7573,24 +7570,24 @@
         <v>8</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>280</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>791</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="E29" s="1" t="s">
         <v>792</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>793</v>
       </c>
       <c r="F29" s="5" t="s">
         <v>413</v>
@@ -7599,21 +7596,21 @@
         <v>8</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>283</v>
       </c>
       <c r="C30" s="1" t="s">
+        <v>795</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>796</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>797</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>679</v>
@@ -7623,48 +7620,48 @@
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>286</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>799</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>800</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E31" s="1" t="s">
         <v>801</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>802</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>671</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>289</v>
       </c>
       <c r="C32" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>805</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>806</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>807</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>413</v>
@@ -7673,7 +7670,7 @@
         <v>8</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
     </row>
   </sheetData>
@@ -7694,13 +7691,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>809</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
+      <c r="A1" s="14" t="s">
+        <v>808</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -7733,10 +7730,10 @@
     </row>
     <row r="5" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
+        <v>809</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>810</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>811</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -7751,19 +7748,19 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>812</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>813</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>814</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>815</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
@@ -7771,16 +7768,16 @@
         <v>1</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>817</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>818</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>819</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -7788,16 +7785,16 @@
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>821</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>823</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>824</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -7805,16 +7802,16 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>825</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>826</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>827</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>828</v>
       </c>
     </row>
   </sheetData>
@@ -7837,16 +7834,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
-        <v>829</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="14"/>
+      <c r="A1" s="14" t="s">
+        <v>828</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -7891,7 +7888,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -7914,12 +7911,12 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -7940,16 +7937,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>832</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>833</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>397</v>
@@ -7961,7 +7958,7 @@
         <v>399</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -8045,7 +8042,7 @@
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="C13" s="1">
         <v>73</v>
@@ -8079,25 +8076,25 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1">
         <v>100</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1">
@@ -8105,12 +8102,12 @@
         <v>96.05263157894737</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -8144,86 +8141,86 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
+        <v>840</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>841</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>842</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>843</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>845</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>846</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>849</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>850</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>851</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>852</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -8231,13 +8228,13 @@
         <v>353</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>854</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>855</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -8245,13 +8242,13 @@
         <v>353</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>856</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -8259,13 +8256,13 @@
         <v>353</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -8273,13 +8270,13 @@
         <v>366</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>858</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>859</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -8287,13 +8284,13 @@
         <v>366</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>861</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>862</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.35">
@@ -8301,13 +8298,13 @@
         <v>375</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -8315,13 +8312,13 @@
         <v>375</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>413</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -8329,13 +8326,13 @@
         <v>375</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>865</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>866</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -8343,13 +8340,13 @@
         <v>375</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>867</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>